<commit_message>
Pin H2KG 2.3 comparator evidence
</commit_message>
<xml_diff>
--- a/ontology_release/output/docs/evaluation/focused_comparator_matrix.xlsx
+++ b/ontology_release/output/docs/evaluation/focused_comparator_matrix.xlsx
@@ -1663,12 +1663,12 @@
     <col width="13" customWidth="1" min="1" max="1"/>
     <col width="55" customWidth="1" min="2" max="2"/>
     <col width="12" customWidth="1" min="3" max="3"/>
-    <col width="51" customWidth="1" min="4" max="4"/>
+    <col width="38" customWidth="1" min="4" max="4"/>
     <col width="12" customWidth="1" min="5" max="5"/>
     <col width="50" customWidth="1" min="6" max="6"/>
     <col width="55" customWidth="1" min="7" max="7"/>
     <col width="42" customWidth="1" min="8" max="8"/>
-    <col width="51" customWidth="1" min="9" max="9"/>
+    <col width="38" customWidth="1" min="9" max="9"/>
     <col width="55" customWidth="1" min="10" max="10"/>
     <col width="14" customWidth="1" min="11" max="11"/>
     <col width="14" customWidth="1" min="12" max="12"/>
@@ -1814,7 +1814,7 @@
       </c>
       <c r="D3" s="2" t="inlineStr">
         <is>
-          <t>odk/src/ontology/mirror/emmo-electrochemistry.owl</t>
+          <t>input/comparators/edo-0.39.0.owl</t>
         </is>
       </c>
       <c r="E3" s="2" t="inlineStr">
@@ -1839,7 +1839,7 @@
       </c>
       <c r="I3" s="2" t="inlineStr">
         <is>
-          <t>odk/src/ontology/mirror/emmo-electrochemistry.owl</t>
+          <t>input/comparators/edo-0.39.0.owl</t>
         </is>
       </c>
       <c r="J3" s="2" t="inlineStr">
@@ -1874,7 +1874,7 @@
       </c>
       <c r="D4" s="2" t="inlineStr">
         <is>
-          <t>odk/src/ontology/mirror/hdo.owl</t>
+          <t>input/comparators/hdo-2026-09-25.owl</t>
         </is>
       </c>
       <c r="E4" s="2" t="inlineStr">
@@ -1899,7 +1899,7 @@
       </c>
       <c r="I4" s="2" t="inlineStr">
         <is>
-          <t>odk/src/ontology/mirror/hdo.owl</t>
+          <t>input/comparators/hdo-2026-09-25.owl</t>
         </is>
       </c>
       <c r="J4" s="2" t="inlineStr">

</xml_diff>